<commit_message>
Pump Ingestion: upload template + flow match the EC/Serial ERP format
Template + PumpUploadBox + uploadPumps now use the export's columns (CUST, CUST_NAME, EC_NO, SO_NO, PUMP_SL_NO, PUMP_MODEL_AS_NAME_PLATE, LIQUID, CAPACITY, HEAD). CUST is reversed to the portal client code for matching; upserts key on serial so re-uploads correct existing pumps in place. Admin page shows SO No (Year/Qty dropped).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/pump_upload_template.xlsx
+++ b/public/pump_upload_template.xlsx
@@ -397,101 +397,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:I2"/>
   <cols>
-    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Client Code</v>
+        <v>CUST</v>
       </c>
       <c r="B1" t="str">
-        <v>Client Name</v>
+        <v>CUST_NAME</v>
       </c>
       <c r="C1" t="str">
-        <v>Model</v>
+        <v>EC_NO</v>
       </c>
       <c r="D1" t="str">
-        <v>Quantity</v>
+        <v>SO_NO</v>
       </c>
       <c r="E1" t="str">
-        <v>SR No</v>
+        <v>PUMP_SL_NO</v>
       </c>
       <c r="F1" t="str">
-        <v>EC No</v>
+        <v>PUMP_MODEL_AS_NAME_PLATE</v>
       </c>
       <c r="G1" t="str">
-        <v>EC Date</v>
+        <v>LIQUID</v>
       </c>
       <c r="H1" t="str">
-        <v>SO Date</v>
+        <v>CAPACITY</v>
       </c>
       <c r="I1" t="str">
-        <v>Liquid</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Capacity</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Head</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Supplier</v>
+        <v>HEAD</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ABCD01X001</v>
+        <v>A00101HOSH</v>
       </c>
       <c r="B2" t="str">
-        <v>Example Sugar Mill Pvt Ltd</v>
+        <v>A. B. SUGARS LTD</v>
       </c>
       <c r="C2" t="str">
-        <v>PCP MX-80</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
+        <v>EC/26/1/180/37619</v>
+      </c>
+      <c r="D2" t="str">
+        <v>SO26/1/180</v>
       </c>
       <c r="E2" t="str">
-        <v>SR-2026-0001</v>
+        <v>25-26/1/1188</v>
       </c>
       <c r="F2" t="str">
-        <v>EC-2026-0001</v>
+        <v>RMOH81100AABN</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-06-15</v>
+        <v>A Heavy Molasses</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-05-20</v>
+        <v>50 m3/hr</v>
       </c>
       <c r="I2" t="str">
-        <v>Spent Wash</v>
-      </c>
-      <c r="J2" t="str">
-        <v>50 m3/hr</v>
-      </c>
-      <c r="K2" t="str">
-        <v>30 m</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Risansi Industries Ltd</v>
+        <v>60 MWC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>